<commit_message>
Alterações e adição do .qmd da análise de correlação
</commit_message>
<xml_diff>
--- a/f2_tabelas/matriz_correlacao.xlsx
+++ b/f2_tabelas/matriz_correlacao.xlsx
@@ -407,7 +407,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>porc_pre_natal_precose</t>
+          <t>porc_pre_natal_precoce</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -843,7 +843,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>porc_pre_natal_precose</t>
+          <t>porc_pre_natal_precoce</t>
         </is>
       </c>
       <c r="B11">

</xml_diff>